<commit_message>
updated customers and line items
</commit_message>
<xml_diff>
--- a/data_full/Employees.xlsx
+++ b/data_full/Employees.xlsx
@@ -22,16 +22,13 @@
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="167" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -42,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -50,21 +47,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -432,61 +420,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K82"/>
+  <dimension ref="A1:K77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>EmployeeID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>FName</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>LName</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>gender</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>SkillsTraining</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>SalesmanshipTraining</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>ProductTraining</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>DOB</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>StartDate</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>TerminationDate</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>LocationID</t>
         </is>
@@ -520,13 +508,13 @@
       <c r="G2" t="b">
         <v>0</v>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>35298</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="I2" s="2" t="n">
         <v>42737</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="J2" s="2" t="n">
         <v>43773</v>
       </c>
       <c r="K2" t="inlineStr">
@@ -563,10 +551,10 @@
       <c r="G3" t="b">
         <v>1</v>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="1" t="n">
         <v>35646</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="I3" s="2" t="n">
         <v>42740</v>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -604,13 +592,13 @@
       <c r="G4" t="b">
         <v>0</v>
       </c>
-      <c r="H4" s="2" t="n">
+      <c r="H4" s="1" t="n">
         <v>34005</v>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="I4" s="2" t="n">
         <v>42737</v>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="J4" s="2" t="n">
         <v>42903</v>
       </c>
       <c r="K4" t="inlineStr">
@@ -647,10 +635,10 @@
       <c r="G5" t="b">
         <v>0</v>
       </c>
-      <c r="H5" s="2" t="n">
+      <c r="H5" s="1" t="n">
         <v>33236</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="I5" s="2" t="n">
         <v>42904</v>
       </c>
       <c r="J5" t="inlineStr"/>
@@ -688,13 +676,13 @@
       <c r="G6" t="b">
         <v>1</v>
       </c>
-      <c r="H6" s="2" t="n">
+      <c r="H6" s="1" t="n">
         <v>35282</v>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="I6" s="2" t="n">
         <v>43774</v>
       </c>
-      <c r="J6" s="3" t="n">
+      <c r="J6" s="2" t="n">
         <v>44122</v>
       </c>
       <c r="K6" t="inlineStr">
@@ -731,10 +719,10 @@
       <c r="G7" t="b">
         <v>0</v>
       </c>
-      <c r="H7" s="2" t="n">
+      <c r="H7" s="1" t="n">
         <v>33036</v>
       </c>
-      <c r="I7" s="3" t="n">
+      <c r="I7" s="2" t="n">
         <v>44123</v>
       </c>
       <c r="J7" t="inlineStr"/>
@@ -772,13 +760,13 @@
       <c r="G8" t="b">
         <v>0</v>
       </c>
-      <c r="H8" s="2" t="n">
+      <c r="H8" s="1" t="n">
         <v>33851</v>
       </c>
-      <c r="I8" s="3" t="n">
+      <c r="I8" s="2" t="n">
         <v>43101</v>
       </c>
-      <c r="J8" s="3" t="n">
+      <c r="J8" s="2" t="n">
         <v>43459</v>
       </c>
       <c r="K8" t="inlineStr">
@@ -815,10 +803,10 @@
       <c r="G9" t="b">
         <v>0</v>
       </c>
-      <c r="H9" s="2" t="n">
+      <c r="H9" s="1" t="n">
         <v>33903</v>
       </c>
-      <c r="I9" s="3" t="n">
+      <c r="I9" s="2" t="n">
         <v>43107</v>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -856,13 +844,13 @@
       <c r="G10" t="b">
         <v>0</v>
       </c>
-      <c r="H10" s="2" t="n">
+      <c r="H10" s="1" t="n">
         <v>34785</v>
       </c>
-      <c r="I10" s="3" t="n">
+      <c r="I10" s="2" t="n">
         <v>43101</v>
       </c>
-      <c r="J10" s="3" t="n">
+      <c r="J10" s="2" t="n">
         <v>43417</v>
       </c>
       <c r="K10" t="inlineStr">
@@ -899,13 +887,13 @@
       <c r="G11" t="b">
         <v>0</v>
       </c>
-      <c r="H11" s="2" t="n">
+      <c r="H11" s="1" t="n">
         <v>34259</v>
       </c>
-      <c r="I11" s="3" t="n">
+      <c r="I11" s="2" t="n">
         <v>43471</v>
       </c>
-      <c r="J11" s="3" t="n">
+      <c r="J11" s="2" t="n">
         <v>43646</v>
       </c>
       <c r="K11" t="inlineStr">
@@ -942,13 +930,13 @@
       <c r="G12" t="b">
         <v>1</v>
       </c>
-      <c r="H12" s="2" t="n">
+      <c r="H12" s="1" t="n">
         <v>35598</v>
       </c>
-      <c r="I12" s="3" t="n">
+      <c r="I12" s="2" t="n">
         <v>43418</v>
       </c>
-      <c r="J12" s="3" t="n">
+      <c r="J12" s="2" t="n">
         <v>44463</v>
       </c>
       <c r="K12" t="inlineStr">
@@ -985,10 +973,10 @@
       <c r="G13" t="b">
         <v>1</v>
       </c>
-      <c r="H13" s="2" t="n">
+      <c r="H13" s="1" t="n">
         <v>35061</v>
       </c>
-      <c r="I13" s="3" t="n">
+      <c r="I13" s="2" t="n">
         <v>43647</v>
       </c>
       <c r="J13" t="inlineStr"/>
@@ -1026,10 +1014,10 @@
       <c r="G14" t="b">
         <v>1</v>
       </c>
-      <c r="H14" s="2" t="n">
+      <c r="H14" s="1" t="n">
         <v>35004</v>
       </c>
-      <c r="I14" s="3" t="n">
+      <c r="I14" s="2" t="n">
         <v>44464</v>
       </c>
       <c r="J14" t="inlineStr"/>
@@ -1067,13 +1055,13 @@
       <c r="G15" t="b">
         <v>1</v>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="H15" s="1" t="n">
         <v>34590</v>
       </c>
-      <c r="I15" s="3" t="n">
+      <c r="I15" s="2" t="n">
         <v>43102</v>
       </c>
-      <c r="J15" s="3" t="n">
+      <c r="J15" s="2" t="n">
         <v>43319</v>
       </c>
       <c r="K15" t="inlineStr">
@@ -1110,13 +1098,13 @@
       <c r="G16" t="b">
         <v>1</v>
       </c>
-      <c r="H16" s="2" t="n">
+      <c r="H16" s="1" t="n">
         <v>33570</v>
       </c>
-      <c r="I16" s="3" t="n">
+      <c r="I16" s="2" t="n">
         <v>43102</v>
       </c>
-      <c r="J16" s="3" t="n">
+      <c r="J16" s="2" t="n">
         <v>43393</v>
       </c>
       <c r="K16" t="inlineStr">
@@ -1153,10 +1141,10 @@
       <c r="G17" t="b">
         <v>1</v>
       </c>
-      <c r="H17" s="2" t="n">
+      <c r="H17" s="1" t="n">
         <v>34642</v>
       </c>
-      <c r="I17" s="3" t="n">
+      <c r="I17" s="2" t="n">
         <v>43103</v>
       </c>
       <c r="J17" t="inlineStr"/>
@@ -1194,13 +1182,13 @@
       <c r="G18" t="b">
         <v>1</v>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="H18" s="1" t="n">
         <v>34301</v>
       </c>
-      <c r="I18" s="3" t="n">
+      <c r="I18" s="2" t="n">
         <v>43320</v>
       </c>
-      <c r="J18" s="3" t="n">
+      <c r="J18" s="2" t="n">
         <v>44270</v>
       </c>
       <c r="K18" t="inlineStr">
@@ -1237,13 +1225,13 @@
       <c r="G19" t="b">
         <v>1</v>
       </c>
-      <c r="H19" s="2" t="n">
+      <c r="H19" s="1" t="n">
         <v>34725</v>
       </c>
-      <c r="I19" s="3" t="n">
+      <c r="I19" s="2" t="n">
         <v>43394</v>
       </c>
-      <c r="J19" s="3" t="n">
+      <c r="J19" s="2" t="n">
         <v>43587</v>
       </c>
       <c r="K19" t="inlineStr">
@@ -1280,10 +1268,10 @@
       <c r="G20" t="b">
         <v>0</v>
       </c>
-      <c r="H20" s="2" t="n">
+      <c r="H20" s="1" t="n">
         <v>33575</v>
       </c>
-      <c r="I20" s="3" t="n">
+      <c r="I20" s="2" t="n">
         <v>43587</v>
       </c>
       <c r="J20" t="inlineStr"/>
@@ -1321,10 +1309,10 @@
       <c r="G21" t="b">
         <v>0</v>
       </c>
-      <c r="H21" s="2" t="n">
+      <c r="H21" s="1" t="n">
         <v>33559</v>
       </c>
-      <c r="I21" s="3" t="n">
+      <c r="I21" s="2" t="n">
         <v>44271</v>
       </c>
       <c r="J21" t="inlineStr"/>
@@ -1362,13 +1350,13 @@
       <c r="G22" t="b">
         <v>0</v>
       </c>
-      <c r="H22" s="2" t="n">
+      <c r="H22" s="1" t="n">
         <v>33632</v>
       </c>
-      <c r="I22" s="3" t="n">
+      <c r="I22" s="2" t="n">
         <v>43471</v>
       </c>
-      <c r="J22" s="3" t="n">
+      <c r="J22" s="2" t="n">
         <v>44515</v>
       </c>
       <c r="K22" t="inlineStr">
@@ -1405,10 +1393,10 @@
       <c r="G23" t="b">
         <v>0</v>
       </c>
-      <c r="H23" s="2" t="n">
+      <c r="H23" s="1" t="n">
         <v>35241</v>
       </c>
-      <c r="I23" s="3" t="n">
+      <c r="I23" s="2" t="n">
         <v>43466</v>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -1446,13 +1434,13 @@
       <c r="G24" t="b">
         <v>0</v>
       </c>
-      <c r="H24" s="2" t="n">
+      <c r="H24" s="1" t="n">
         <v>33389</v>
       </c>
-      <c r="I24" s="3" t="n">
+      <c r="I24" s="2" t="n">
         <v>43467</v>
       </c>
-      <c r="J24" s="3" t="n">
+      <c r="J24" s="2" t="n">
         <v>44392</v>
       </c>
       <c r="K24" t="inlineStr">
@@ -1489,10 +1477,10 @@
       <c r="G25" t="b">
         <v>0</v>
       </c>
-      <c r="H25" s="2" t="n">
+      <c r="H25" s="1" t="n">
         <v>34769</v>
       </c>
-      <c r="I25" s="3" t="n">
+      <c r="I25" s="2" t="n">
         <v>43833</v>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -1530,10 +1518,10 @@
       <c r="G26" t="b">
         <v>1</v>
       </c>
-      <c r="H26" s="2" t="n">
+      <c r="H26" s="1" t="n">
         <v>33077</v>
       </c>
-      <c r="I26" s="3" t="n">
+      <c r="I26" s="2" t="n">
         <v>44393</v>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -1571,13 +1559,13 @@
       <c r="G27" t="b">
         <v>1</v>
       </c>
-      <c r="H27" s="2" t="n">
+      <c r="H27" s="1" t="n">
         <v>33539</v>
       </c>
-      <c r="I27" s="3" t="n">
+      <c r="I27" s="2" t="n">
         <v>43471</v>
       </c>
-      <c r="J27" s="3" t="n">
+      <c r="J27" s="2" t="n">
         <v>44410</v>
       </c>
       <c r="K27" t="inlineStr">
@@ -1614,13 +1602,13 @@
       <c r="G28" t="b">
         <v>1</v>
       </c>
-      <c r="H28" s="2" t="n">
+      <c r="H28" s="1" t="n">
         <v>33194</v>
       </c>
-      <c r="I28" s="3" t="n">
+      <c r="I28" s="2" t="n">
         <v>43478</v>
       </c>
-      <c r="J28" s="3" t="n">
+      <c r="J28" s="2" t="n">
         <v>43601</v>
       </c>
       <c r="K28" t="inlineStr">
@@ -1657,10 +1645,10 @@
       <c r="G29" t="b">
         <v>0</v>
       </c>
-      <c r="H29" s="2" t="n">
+      <c r="H29" s="1" t="n">
         <v>35804</v>
       </c>
-      <c r="I29" s="3" t="n">
+      <c r="I29" s="2" t="n">
         <v>43469</v>
       </c>
       <c r="J29" t="inlineStr"/>
@@ -1698,13 +1686,13 @@
       <c r="G30" t="b">
         <v>0</v>
       </c>
-      <c r="H30" s="2" t="n">
+      <c r="H30" s="1" t="n">
         <v>33042</v>
       </c>
-      <c r="I30" s="3" t="n">
+      <c r="I30" s="2" t="n">
         <v>43602</v>
       </c>
-      <c r="J30" s="3" t="n">
+      <c r="J30" s="2" t="n">
         <v>44193</v>
       </c>
       <c r="K30" t="inlineStr">
@@ -1741,10 +1729,10 @@
       <c r="G31" t="b">
         <v>0</v>
       </c>
-      <c r="H31" s="2" t="n">
+      <c r="H31" s="1" t="n">
         <v>34836</v>
       </c>
-      <c r="I31" s="3" t="n">
+      <c r="I31" s="2" t="n">
         <v>44198</v>
       </c>
       <c r="J31" t="inlineStr"/>
@@ -1782,10 +1770,10 @@
       <c r="G32" t="b">
         <v>1</v>
       </c>
-      <c r="H32" s="2" t="n">
+      <c r="H32" s="1" t="n">
         <v>34250</v>
       </c>
-      <c r="I32" s="3" t="n">
+      <c r="I32" s="2" t="n">
         <v>44411</v>
       </c>
       <c r="J32" t="inlineStr"/>
@@ -1823,13 +1811,13 @@
       <c r="G33" t="b">
         <v>0</v>
       </c>
-      <c r="H33" s="2" t="n">
+      <c r="H33" s="1" t="n">
         <v>33427</v>
       </c>
-      <c r="I33" s="3" t="n">
+      <c r="I33" s="2" t="n">
         <v>43838</v>
       </c>
-      <c r="J33" s="3" t="n">
+      <c r="J33" s="2" t="n">
         <v>44477</v>
       </c>
       <c r="K33" t="inlineStr">
@@ -1866,10 +1854,10 @@
       <c r="G34" t="b">
         <v>0</v>
       </c>
-      <c r="H34" s="2" t="n">
+      <c r="H34" s="1" t="n">
         <v>35323</v>
       </c>
-      <c r="I34" s="3" t="n">
+      <c r="I34" s="2" t="n">
         <v>43834</v>
       </c>
       <c r="J34" t="inlineStr"/>
@@ -1907,10 +1895,10 @@
       <c r="G35" t="b">
         <v>0</v>
       </c>
-      <c r="H35" s="2" t="n">
+      <c r="H35" s="1" t="n">
         <v>35375</v>
       </c>
-      <c r="I35" s="3" t="n">
+      <c r="I35" s="2" t="n">
         <v>43832</v>
       </c>
       <c r="J35" t="inlineStr"/>
@@ -1948,10 +1936,10 @@
       <c r="G36" t="b">
         <v>1</v>
       </c>
-      <c r="H36" s="2" t="n">
+      <c r="H36" s="1" t="n">
         <v>35521</v>
       </c>
-      <c r="I36" s="3" t="n">
+      <c r="I36" s="2" t="n">
         <v>44478</v>
       </c>
       <c r="J36" t="inlineStr"/>
@@ -1989,10 +1977,10 @@
       <c r="G37" t="b">
         <v>0</v>
       </c>
-      <c r="H37" s="2" t="n">
+      <c r="H37" s="1" t="n">
         <v>33252</v>
       </c>
-      <c r="I37" s="3" t="n">
+      <c r="I37" s="2" t="n">
         <v>43831</v>
       </c>
       <c r="J37" t="inlineStr"/>
@@ -2030,13 +2018,13 @@
       <c r="G38" t="b">
         <v>1</v>
       </c>
-      <c r="H38" s="2" t="n">
+      <c r="H38" s="1" t="n">
         <v>33089</v>
       </c>
-      <c r="I38" s="3" t="n">
+      <c r="I38" s="2" t="n">
         <v>43835</v>
       </c>
-      <c r="J38" s="3" t="n">
+      <c r="J38" s="2" t="n">
         <v>43927</v>
       </c>
       <c r="K38" t="inlineStr">
@@ -2073,10 +2061,10 @@
       <c r="G39" t="b">
         <v>1</v>
       </c>
-      <c r="H39" s="2" t="n">
+      <c r="H39" s="1" t="n">
         <v>33255</v>
       </c>
-      <c r="I39" s="3" t="n">
+      <c r="I39" s="2" t="n">
         <v>43831</v>
       </c>
       <c r="J39" t="inlineStr"/>
@@ -2114,13 +2102,13 @@
       <c r="G40" t="b">
         <v>0</v>
       </c>
-      <c r="H40" s="2" t="n">
+      <c r="H40" s="1" t="n">
         <v>33401</v>
       </c>
-      <c r="I40" s="3" t="n">
+      <c r="I40" s="2" t="n">
         <v>43928</v>
       </c>
-      <c r="J40" s="3" t="n">
+      <c r="J40" s="2" t="n">
         <v>44501</v>
       </c>
       <c r="K40" t="inlineStr">
@@ -2157,10 +2145,10 @@
       <c r="G41" t="b">
         <v>1</v>
       </c>
-      <c r="H41" s="2" t="n">
+      <c r="H41" s="1" t="n">
         <v>33238</v>
       </c>
-      <c r="I41" s="3" t="n">
+      <c r="I41" s="2" t="n">
         <v>44502</v>
       </c>
       <c r="J41" t="inlineStr"/>
@@ -2198,10 +2186,10 @@
       <c r="G42" t="b">
         <v>1</v>
       </c>
-      <c r="H42" s="2" t="n">
+      <c r="H42" s="1" t="n">
         <v>33627</v>
       </c>
-      <c r="I42" s="3" t="n">
+      <c r="I42" s="2" t="n">
         <v>43831</v>
       </c>
       <c r="J42" t="inlineStr"/>
@@ -2239,13 +2227,13 @@
       <c r="G43" t="b">
         <v>1</v>
       </c>
-      <c r="H43" s="2" t="n">
+      <c r="H43" s="1" t="n">
         <v>34008</v>
       </c>
-      <c r="I43" s="3" t="n">
+      <c r="I43" s="2" t="n">
         <v>43833</v>
       </c>
-      <c r="J43" s="3" t="n">
+      <c r="J43" s="2" t="n">
         <v>44455</v>
       </c>
       <c r="K43" t="inlineStr">
@@ -2282,13 +2270,13 @@
       <c r="G44" t="b">
         <v>1</v>
       </c>
-      <c r="H44" s="2" t="n">
+      <c r="H44" s="1" t="n">
         <v>33265</v>
       </c>
-      <c r="I44" s="3" t="n">
+      <c r="I44" s="2" t="n">
         <v>43831</v>
       </c>
-      <c r="J44" s="3" t="n">
+      <c r="J44" s="2" t="n">
         <v>44045</v>
       </c>
       <c r="K44" t="inlineStr">
@@ -2325,10 +2313,10 @@
       <c r="G45" t="b">
         <v>1</v>
       </c>
-      <c r="H45" s="2" t="n">
+      <c r="H45" s="1" t="n">
         <v>35057</v>
       </c>
-      <c r="I45" s="3" t="n">
+      <c r="I45" s="2" t="n">
         <v>44046</v>
       </c>
       <c r="J45" t="inlineStr"/>
@@ -2366,10 +2354,10 @@
       <c r="G46" t="b">
         <v>1</v>
       </c>
-      <c r="H46" s="2" t="n">
+      <c r="H46" s="1" t="n">
         <v>33548</v>
       </c>
-      <c r="I46" s="3" t="n">
+      <c r="I46" s="2" t="n">
         <v>44456</v>
       </c>
       <c r="J46" t="inlineStr"/>
@@ -2407,10 +2395,10 @@
       <c r="G47" t="b">
         <v>0</v>
       </c>
-      <c r="H47" s="2" t="n">
+      <c r="H47" s="1" t="n">
         <v>35278</v>
       </c>
-      <c r="I47" s="3" t="n">
+      <c r="I47" s="2" t="n">
         <v>44197</v>
       </c>
       <c r="J47" t="inlineStr"/>
@@ -2448,10 +2436,10 @@
       <c r="G48" t="b">
         <v>1</v>
       </c>
-      <c r="H48" s="2" t="n">
+      <c r="H48" s="1" t="n">
         <v>34963</v>
       </c>
-      <c r="I48" s="3" t="n">
+      <c r="I48" s="2" t="n">
         <v>44201</v>
       </c>
       <c r="J48" t="inlineStr"/>
@@ -2489,10 +2477,10 @@
       <c r="G49" t="b">
         <v>1</v>
       </c>
-      <c r="H49" s="2" t="n">
+      <c r="H49" s="1" t="n">
         <v>35224</v>
       </c>
-      <c r="I49" s="3" t="n">
+      <c r="I49" s="2" t="n">
         <v>44198</v>
       </c>
       <c r="J49" t="inlineStr"/>
@@ -2530,10 +2518,10 @@
       <c r="G50" t="b">
         <v>1</v>
       </c>
-      <c r="H50" s="2" t="n">
+      <c r="H50" s="1" t="n">
         <v>33172</v>
       </c>
-      <c r="I50" s="3" t="n">
+      <c r="I50" s="2" t="n">
         <v>44197</v>
       </c>
       <c r="J50" t="inlineStr"/>
@@ -2571,13 +2559,13 @@
       <c r="G51" t="b">
         <v>1</v>
       </c>
-      <c r="H51" s="2" t="n">
+      <c r="H51" s="1" t="n">
         <v>35356</v>
       </c>
-      <c r="I51" s="3" t="n">
+      <c r="I51" s="2" t="n">
         <v>44202</v>
       </c>
-      <c r="J51" s="3" t="n">
+      <c r="J51" s="2" t="n">
         <v>44444</v>
       </c>
       <c r="K51" t="inlineStr">
@@ -2614,10 +2602,10 @@
       <c r="G52" t="b">
         <v>1</v>
       </c>
-      <c r="H52" s="2" t="n">
+      <c r="H52" s="1" t="n">
         <v>33722</v>
       </c>
-      <c r="I52" s="3" t="n">
+      <c r="I52" s="2" t="n">
         <v>44202</v>
       </c>
       <c r="J52" t="inlineStr"/>
@@ -2655,10 +2643,10 @@
       <c r="G53" t="b">
         <v>0</v>
       </c>
-      <c r="H53" s="2" t="n">
+      <c r="H53" s="1" t="n">
         <v>33374</v>
       </c>
-      <c r="I53" s="3" t="n">
+      <c r="I53" s="2" t="n">
         <v>44445</v>
       </c>
       <c r="J53" t="inlineStr"/>
@@ -2696,10 +2684,10 @@
       <c r="G54" t="b">
         <v>1</v>
       </c>
-      <c r="H54" s="2" t="n">
+      <c r="H54" s="1" t="n">
         <v>33634</v>
       </c>
-      <c r="I54" s="3" t="n">
+      <c r="I54" s="2" t="n">
         <v>44197</v>
       </c>
       <c r="J54" t="inlineStr"/>
@@ -2737,10 +2725,10 @@
       <c r="G55" t="b">
         <v>1</v>
       </c>
-      <c r="H55" s="2" t="n">
+      <c r="H55" s="1" t="n">
         <v>33113</v>
       </c>
-      <c r="I55" s="3" t="n">
+      <c r="I55" s="2" t="n">
         <v>44197</v>
       </c>
       <c r="J55" t="inlineStr"/>
@@ -2778,10 +2766,10 @@
       <c r="G56" t="b">
         <v>0</v>
       </c>
-      <c r="H56" s="2" t="n">
+      <c r="H56" s="1" t="n">
         <v>33997</v>
       </c>
-      <c r="I56" s="3" t="n">
+      <c r="I56" s="2" t="n">
         <v>44201</v>
       </c>
       <c r="J56" t="inlineStr"/>
@@ -2797,21 +2785,21 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Cody</t>
+          <t>Ashley</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Wu</t>
+          <t>Fletcher</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="E57" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F57" t="b">
         <v>1</v>
@@ -2819,11 +2807,11 @@
       <c r="G57" t="b">
         <v>0</v>
       </c>
-      <c r="H57" s="2" t="n">
-        <v>30441</v>
-      </c>
-      <c r="I57" s="3" t="n">
-        <v>44565</v>
+      <c r="H57" s="1" t="n">
+        <v>37096</v>
+      </c>
+      <c r="I57" s="2" t="n">
+        <v>44564</v>
       </c>
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr">
@@ -2838,33 +2826,33 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Brian</t>
+          <t>Lori</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Roy</t>
+          <t>Beck</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="E58" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F58" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G58" t="b">
-        <v>0</v>
-      </c>
-      <c r="H58" s="2" t="n">
-        <v>33690</v>
-      </c>
-      <c r="I58" s="3" t="n">
-        <v>44562</v>
+        <v>1</v>
+      </c>
+      <c r="H58" s="1" t="n">
+        <v>38155</v>
+      </c>
+      <c r="I58" s="2" t="n">
+        <v>44563</v>
       </c>
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
@@ -2879,32 +2867,32 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Robin</t>
+          <t>Patricia</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Johnson</t>
+          <t>Wagner</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="E59" t="b">
         <v>1</v>
       </c>
       <c r="F59" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G59" t="b">
-        <v>0</v>
-      </c>
-      <c r="H59" s="2" t="n">
-        <v>36970</v>
-      </c>
-      <c r="I59" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H59" s="1" t="n">
+        <v>34984</v>
+      </c>
+      <c r="I59" s="2" t="n">
         <v>44564</v>
       </c>
       <c r="J59" t="inlineStr"/>
@@ -2920,12 +2908,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Matthew</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Castro</t>
+          <t>Gomez</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2934,7 +2922,7 @@
         </is>
       </c>
       <c r="E60" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F60" t="b">
         <v>1</v>
@@ -2942,11 +2930,11 @@
       <c r="G60" t="b">
         <v>1</v>
       </c>
-      <c r="H60" s="2" t="n">
-        <v>32978</v>
-      </c>
-      <c r="I60" s="3" t="n">
-        <v>44564</v>
+      <c r="H60" s="1" t="n">
+        <v>30944</v>
+      </c>
+      <c r="I60" s="2" t="n">
+        <v>44562</v>
       </c>
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr">
@@ -2961,32 +2949,32 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Stephanie</t>
+          <t>Glenn</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Cortez</t>
+          <t>Jones</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="E61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F61" t="b">
         <v>1</v>
       </c>
       <c r="G61" t="b">
-        <v>1</v>
-      </c>
-      <c r="H61" s="2" t="n">
-        <v>27735</v>
-      </c>
-      <c r="I61" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" s="1" t="n">
+        <v>38024</v>
+      </c>
+      <c r="I61" s="2" t="n">
         <v>44564</v>
       </c>
       <c r="J61" t="inlineStr"/>
@@ -3002,12 +2990,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Matthew</t>
+          <t>Corey</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Gomez</t>
+          <t>Jones</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3016,19 +3004,19 @@
         </is>
       </c>
       <c r="E62" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F62" t="b">
         <v>0</v>
       </c>
       <c r="G62" t="b">
-        <v>1</v>
-      </c>
-      <c r="H62" s="2" t="n">
-        <v>32483</v>
-      </c>
-      <c r="I62" s="3" t="n">
-        <v>44929</v>
+        <v>0</v>
+      </c>
+      <c r="H62" s="1" t="n">
+        <v>35659</v>
+      </c>
+      <c r="I62" s="2" t="n">
+        <v>44930</v>
       </c>
       <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr">
@@ -3043,17 +3031,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Sara</t>
+          <t>Mark</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Carroll</t>
+          <t>West</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="E63" t="b">
@@ -3063,13 +3051,13 @@
         <v>0</v>
       </c>
       <c r="G63" t="b">
-        <v>0</v>
-      </c>
-      <c r="H63" s="2" t="n">
-        <v>27973</v>
-      </c>
-      <c r="I63" s="3" t="n">
-        <v>44927</v>
+        <v>1</v>
+      </c>
+      <c r="H63" s="1" t="n">
+        <v>31145</v>
+      </c>
+      <c r="I63" s="2" t="n">
+        <v>44930</v>
       </c>
       <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr">
@@ -3084,12 +3072,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Lori</t>
+          <t>Laura</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Mccoy</t>
+          <t>Perez</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3104,13 +3092,13 @@
         <v>1</v>
       </c>
       <c r="G64" t="b">
-        <v>1</v>
-      </c>
-      <c r="H64" s="2" t="n">
-        <v>32787</v>
-      </c>
-      <c r="I64" s="3" t="n">
-        <v>44928</v>
+        <v>0</v>
+      </c>
+      <c r="H64" s="1" t="n">
+        <v>31440</v>
+      </c>
+      <c r="I64" s="2" t="n">
+        <v>44930</v>
       </c>
       <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr">
@@ -3125,21 +3113,21 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Christian</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Thompson</t>
+          <t>Williams</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="E65" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F65" t="b">
         <v>1</v>
@@ -3147,10 +3135,10 @@
       <c r="G65" t="b">
         <v>1</v>
       </c>
-      <c r="H65" s="2" t="n">
-        <v>31078</v>
-      </c>
-      <c r="I65" s="3" t="n">
+      <c r="H65" s="1" t="n">
+        <v>29458</v>
+      </c>
+      <c r="I65" s="2" t="n">
         <v>44928</v>
       </c>
       <c r="J65" t="inlineStr"/>
@@ -3166,17 +3154,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Kimberly</t>
+          <t>Robert</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Lane</t>
+          <t>Henry</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="E66" t="b">
@@ -3186,13 +3174,13 @@
         <v>0</v>
       </c>
       <c r="G66" t="b">
-        <v>0</v>
-      </c>
-      <c r="H66" s="2" t="n">
-        <v>36103</v>
-      </c>
-      <c r="I66" s="3" t="n">
-        <v>44929</v>
+        <v>1</v>
+      </c>
+      <c r="H66" s="1" t="n">
+        <v>34252</v>
+      </c>
+      <c r="I66" s="2" t="n">
+        <v>44927</v>
       </c>
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr">
@@ -3207,33 +3195,33 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Emily</t>
+          <t>Chase</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Frost</t>
+          <t>Fuller</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="E67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F67" t="b">
         <v>0</v>
       </c>
       <c r="G67" t="b">
-        <v>0</v>
-      </c>
-      <c r="H67" s="2" t="n">
-        <v>34072</v>
-      </c>
-      <c r="I67" s="3" t="n">
-        <v>45293</v>
+        <v>1</v>
+      </c>
+      <c r="H67" s="1" t="n">
+        <v>37119</v>
+      </c>
+      <c r="I67" s="2" t="n">
+        <v>45294</v>
       </c>
       <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr">
@@ -3248,12 +3236,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Aimee</t>
+          <t>Sarah</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Mendez</t>
+          <t>Kim</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3268,12 +3256,12 @@
         <v>0</v>
       </c>
       <c r="G68" t="b">
-        <v>1</v>
-      </c>
-      <c r="H68" s="2" t="n">
-        <v>34911</v>
-      </c>
-      <c r="I68" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="1" t="n">
+        <v>35404</v>
+      </c>
+      <c r="I68" s="2" t="n">
         <v>45293</v>
       </c>
       <c r="J68" t="inlineStr"/>
@@ -3289,21 +3277,21 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Ricky</t>
+          <t>Bryan</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Sosa</t>
+          <t>Guzman</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="E69" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F69" t="b">
         <v>0</v>
@@ -3311,11 +3299,11 @@
       <c r="G69" t="b">
         <v>0</v>
       </c>
-      <c r="H69" s="2" t="n">
-        <v>32550</v>
-      </c>
-      <c r="I69" s="3" t="n">
-        <v>45293</v>
+      <c r="H69" s="1" t="n">
+        <v>29629</v>
+      </c>
+      <c r="I69" s="2" t="n">
+        <v>45295</v>
       </c>
       <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr">
@@ -3330,33 +3318,33 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Dennis</t>
+          <t>Laura</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Contreras</t>
+          <t>Evans</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="E70" t="b">
         <v>1</v>
       </c>
       <c r="F70" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G70" t="b">
-        <v>0</v>
-      </c>
-      <c r="H70" s="2" t="n">
-        <v>32891</v>
-      </c>
-      <c r="I70" s="3" t="n">
-        <v>45293</v>
+        <v>1</v>
+      </c>
+      <c r="H70" s="1" t="n">
+        <v>36954</v>
+      </c>
+      <c r="I70" s="2" t="n">
+        <v>45294</v>
       </c>
       <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr">
@@ -3371,12 +3359,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Patrick</t>
+          <t>Eddie</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Norris</t>
+          <t>Grimes</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3385,19 +3373,19 @@
         </is>
       </c>
       <c r="E71" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F71" t="b">
         <v>1</v>
       </c>
       <c r="G71" t="b">
-        <v>1</v>
-      </c>
-      <c r="H71" s="2" t="n">
-        <v>29789</v>
-      </c>
-      <c r="I71" s="3" t="n">
-        <v>45293</v>
+        <v>0</v>
+      </c>
+      <c r="H71" s="1" t="n">
+        <v>38208</v>
+      </c>
+      <c r="I71" s="2" t="n">
+        <v>45292</v>
       </c>
       <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr">
@@ -3412,32 +3400,32 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Kayla</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Lewis</t>
+          <t>Johnson</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="E72" t="b">
         <v>0</v>
       </c>
       <c r="F72" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G72" t="b">
         <v>0</v>
       </c>
-      <c r="H72" s="2" t="n">
-        <v>27788</v>
-      </c>
-      <c r="I72" s="3" t="n">
+      <c r="H72" s="1" t="n">
+        <v>29299</v>
+      </c>
+      <c r="I72" s="2" t="n">
         <v>45660</v>
       </c>
       <c r="J72" t="inlineStr"/>
@@ -3453,33 +3441,33 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Carol</t>
+          <t>Nathaniel</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Wheeler</t>
+          <t>Gordon</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="E73" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F73" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G73" t="b">
-        <v>1</v>
-      </c>
-      <c r="H73" s="2" t="n">
-        <v>35683</v>
-      </c>
-      <c r="I73" s="3" t="n">
-        <v>45659</v>
+        <v>0</v>
+      </c>
+      <c r="H73" s="1" t="n">
+        <v>35791</v>
+      </c>
+      <c r="I73" s="2" t="n">
+        <v>45660</v>
       </c>
       <c r="J73" t="inlineStr"/>
       <c r="K73" t="inlineStr">
@@ -3494,33 +3482,33 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Sonya</t>
+          <t>Antonio</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Palmer</t>
+          <t>Foster</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="E74" t="b">
         <v>1</v>
       </c>
       <c r="F74" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G74" t="b">
-        <v>0</v>
-      </c>
-      <c r="H74" s="2" t="n">
-        <v>30348</v>
-      </c>
-      <c r="I74" s="3" t="n">
-        <v>45659</v>
+        <v>1</v>
+      </c>
+      <c r="H74" s="1" t="n">
+        <v>37829</v>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>45658</v>
       </c>
       <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr">
@@ -3535,12 +3523,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Melissa</t>
+          <t>Caitlyn</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Rodriguez</t>
+          <t>Harris</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3557,11 +3545,11 @@
       <c r="G75" t="b">
         <v>1</v>
       </c>
-      <c r="H75" s="2" t="n">
-        <v>29915</v>
-      </c>
-      <c r="I75" s="3" t="n">
-        <v>45660</v>
+      <c r="H75" s="1" t="n">
+        <v>29927</v>
+      </c>
+      <c r="I75" s="2" t="n">
+        <v>45658</v>
       </c>
       <c r="J75" t="inlineStr"/>
       <c r="K75" t="inlineStr">
@@ -3576,17 +3564,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Isabella</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Mcguire</t>
+          <t>Mcmahon</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="E76" t="b">
@@ -3598,11 +3586,11 @@
       <c r="G76" t="b">
         <v>0</v>
       </c>
-      <c r="H76" s="2" t="n">
-        <v>31701</v>
-      </c>
-      <c r="I76" s="3" t="n">
-        <v>45658</v>
+      <c r="H76" s="1" t="n">
+        <v>31920</v>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>45661</v>
       </c>
       <c r="J76" t="inlineStr"/>
       <c r="K76" t="inlineStr">
@@ -3617,12 +3605,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>William</t>
+          <t>Kevin</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Rose</t>
+          <t>Montgomery</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3639,221 +3627,16 @@
       <c r="G77" t="b">
         <v>1</v>
       </c>
-      <c r="H77" s="2" t="n">
-        <v>28961</v>
-      </c>
-      <c r="I77" s="3" t="n">
-        <v>45661</v>
+      <c r="H77" s="1" t="n">
+        <v>37206</v>
+      </c>
+      <c r="I77" s="2" t="n">
+        <v>45659</v>
       </c>
       <c r="J77" t="inlineStr"/>
       <c r="K77" t="inlineStr">
         <is>
           <t>L15</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="n">
-        <v>77</v>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>Kimberly</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Holland</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="E78" t="b">
-        <v>1</v>
-      </c>
-      <c r="F78" t="b">
-        <v>1</v>
-      </c>
-      <c r="G78" t="b">
-        <v>0</v>
-      </c>
-      <c r="H78" s="2" t="n">
-        <v>30570</v>
-      </c>
-      <c r="I78" s="3" t="n">
-        <v>45293</v>
-      </c>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>L14</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="n">
-        <v>78</v>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Micheal</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>Oconnell</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="E79" t="b">
-        <v>1</v>
-      </c>
-      <c r="F79" t="b">
-        <v>1</v>
-      </c>
-      <c r="G79" t="b">
-        <v>0</v>
-      </c>
-      <c r="H79" s="2" t="n">
-        <v>35027</v>
-      </c>
-      <c r="I79" s="3" t="n">
-        <v>45293</v>
-      </c>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>L14</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="n">
-        <v>79</v>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>Charles</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Gonzalez</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="E80" t="b">
-        <v>1</v>
-      </c>
-      <c r="F80" t="b">
-        <v>0</v>
-      </c>
-      <c r="G80" t="b">
-        <v>1</v>
-      </c>
-      <c r="H80" s="2" t="n">
-        <v>27748</v>
-      </c>
-      <c r="I80" s="3" t="n">
-        <v>45293</v>
-      </c>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>L14</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="n">
-        <v>80</v>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Joshua</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>Mcdonald</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="E81" t="b">
-        <v>1</v>
-      </c>
-      <c r="F81" t="b">
-        <v>0</v>
-      </c>
-      <c r="G81" t="b">
-        <v>0</v>
-      </c>
-      <c r="H81" s="2" t="n">
-        <v>30530</v>
-      </c>
-      <c r="I81" s="3" t="n">
-        <v>45293</v>
-      </c>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr">
-        <is>
-          <t>L14</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="n">
-        <v>81</v>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Jennifer</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Sanders</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="E82" t="b">
-        <v>0</v>
-      </c>
-      <c r="F82" t="b">
-        <v>0</v>
-      </c>
-      <c r="G82" t="b">
-        <v>0</v>
-      </c>
-      <c r="H82" s="2" t="n">
-        <v>33118</v>
-      </c>
-      <c r="I82" s="3" t="n">
-        <v>45293</v>
-      </c>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>L14</t>
         </is>
       </c>
     </row>

</xml_diff>